<commit_message>
Refresh derived workbook and integrity manifest
</commit_message>
<xml_diff>
--- a/01_data/Healthcare_Chatbots_Evidence.xlsx
+++ b/01_data/Healthcare_Chatbots_Evidence.xlsx
@@ -15225,7 +15225,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15277,7 +15277,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15381,7 +15381,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15433,7 +15433,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15485,7 +15485,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15537,7 +15537,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15589,7 +15589,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15641,7 +15641,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15693,7 +15693,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15745,11 +15745,11 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="47" customHeight="1">
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">CE06B</t>
@@ -15797,7 +15797,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15901,7 +15901,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -15953,7 +15953,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -16057,7 +16057,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>
@@ -16109,7 +16109,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single AI-assisted analytical workflow; no independent reliability claim</t>
+          <t xml:space="preserve">Single analytical workflow; no independent reliability claim</t>
         </is>
       </c>
     </row>

</xml_diff>